<commit_message>
chore: replace enriched mapping copy with original filename
Renamed fbdi_applaud_mapping_enriched.xlsx back to
fbdi_applaud_mapping.xlsx now that the Excel lock is released.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fbdi_applaud_mapping.xlsx
+++ b/fbdi_applaud_mapping.xlsx
@@ -1169,11 +1169,19 @@
           <t>EGO_CHANGES_INT</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>T_EGO_CHANGES_INT</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>T82</t>
+        </is>
+      </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -1190,11 +1198,19 @@
           <t>EGO_CHANGE_ATTACHMENTS_INT</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>T_EGO_CHANGE_ATTACHMENTS_INT</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>T80</t>
+        </is>
+      </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
@@ -1253,11 +1269,19 @@
           <t>EGO_CHANGE_LINES_INT</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>T_EGO_CHANGE_LINES_INT</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>T81</t>
+        </is>
+      </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr"/>
@@ -1274,11 +1298,19 @@
           <t>EGO_ITEM_INTF_EFF_B</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>T_EGO_ITEM_INTF_EFF_B</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>T86</t>
+        </is>
+      </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
@@ -1316,11 +1348,19 @@
           <t>EGP_COMPONENTS_INTERFACE</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_COMPONENTS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>T91</t>
+        </is>
+      </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr"/>
@@ -1337,11 +1377,19 @@
           <t>EGP_ITEM_ATTACHMENTS_INTF</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_ITEM_ATTACHMENTS_INTF</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>T40</t>
+        </is>
+      </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
@@ -1358,11 +1406,19 @@
           <t>EGP_ITEM_RELATIONSHIPS_INTF</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_ITEM_RELATIONSHIPS_INTF</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>T88</t>
+        </is>
+      </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr"/>
@@ -1400,11 +1456,19 @@
           <t>EGP_REF_DESGS_INTERFACE</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_REF_DESGS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>T93</t>
+        </is>
+      </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr"/>
@@ -1421,11 +1485,19 @@
           <t>EGP_STRUCTURES_INTERFACE</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_STRUCTURES_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>T94</t>
+        </is>
+      </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr"/>
@@ -1442,11 +1514,19 @@
           <t>EGP_SUB_COMPS_INTERFACE</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_SUB_COMPS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>T92</t>
+        </is>
+      </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr"/>
@@ -1463,11 +1543,19 @@
           <t>EGP_SYSTEM_ITEMS_INTERFACE</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr"/>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_SYSTEM_ITEMS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>T90</t>
+        </is>
+      </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr"/>
@@ -1887,11 +1975,19 @@
           <t>HZ_IMP_ACCOUNTS_T</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr"/>
-      <c r="D68" s="4" t="inlineStr"/>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_ACCOUNTS_T</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>T51</t>
+        </is>
+      </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr"/>
@@ -1908,11 +2004,19 @@
           <t>HZ_IMP_ACCTCONTACTS_T</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr"/>
-      <c r="D69" s="4" t="inlineStr"/>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_ACCTCONTACTS_T</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>T70</t>
+        </is>
+      </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr"/>
@@ -1929,11 +2033,19 @@
           <t>HZ_IMP_ACCTSITES_T</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr"/>
-      <c r="D70" s="4" t="inlineStr"/>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_ACCTSITES_T</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>T30</t>
+        </is>
+      </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr"/>
@@ -1950,11 +2062,19 @@
           <t>HZ_IMP_ACCTSITEUSES_T</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr"/>
-      <c r="D71" s="4" t="inlineStr"/>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_ACCTSITEUSES_T</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>T43</t>
+        </is>
+      </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr"/>
@@ -1992,11 +2112,19 @@
           <t>HZ_IMP_CONTACTPTS_T</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr"/>
-      <c r="D73" s="4" t="inlineStr"/>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_CONTACTPTS_T</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>T71</t>
+        </is>
+      </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr"/>
@@ -2013,11 +2141,19 @@
           <t>HZ_IMP_CONTACTROLES</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr"/>
-      <c r="D74" s="4" t="inlineStr"/>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_CONTACTROLES</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>T72</t>
+        </is>
+      </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr"/>
@@ -2034,11 +2170,19 @@
           <t>HZ_IMP_CONTACTS_T</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr"/>
-      <c r="D75" s="4" t="inlineStr"/>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_CONTACTS_T</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>T73</t>
+        </is>
+      </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr"/>
@@ -2055,11 +2199,19 @@
           <t>HZ_IMP_LOCATIONS_T</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr"/>
-      <c r="D76" s="4" t="inlineStr"/>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_LOCATIONS_T</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>T44</t>
+        </is>
+      </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr"/>
@@ -2076,11 +2228,19 @@
           <t>HZ_IMP_PARTIES_T</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr"/>
-      <c r="D77" s="4" t="inlineStr"/>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_PARTIES_T</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>T50</t>
+        </is>
+      </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr"/>
@@ -2118,11 +2278,19 @@
           <t>HZ_IMP_PARTYSITEUSES_T</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr"/>
-      <c r="D79" s="4" t="inlineStr"/>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_PARTYSITEUSES_T</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>T42</t>
+        </is>
+      </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr"/>
@@ -2160,11 +2328,19 @@
           <t>HZ_IMP_RELSHIPS_T</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr"/>
-      <c r="D81" s="4" t="inlineStr"/>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_RELSHIPS_T</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>T74</t>
+        </is>
+      </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr"/>
@@ -2181,11 +2357,19 @@
           <t>HZ_IMP_ROLERESP</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr"/>
-      <c r="D82" s="4" t="inlineStr"/>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>T_HZ_IMP_ROLERESP</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>TC7</t>
+        </is>
+      </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr"/>
@@ -2223,11 +2407,19 @@
           <t>RA_CUSTOMER_PROFILES_INT_ALL</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr"/>
-      <c r="D84" s="4" t="inlineStr"/>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>T_RA_CUSTOMER_PROFILES_INT_ALL</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr"/>
@@ -2370,11 +2562,19 @@
           <t>QP_MATRIX_DIMENSIONS_INT</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr"/>
-      <c r="D91" s="4" t="inlineStr"/>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_MATRIX_DIMENSIONS_INT</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr"/>
@@ -2391,11 +2591,19 @@
           <t>QP_MATRIX_RULES_INT</t>
         </is>
       </c>
-      <c r="C92" s="4" t="inlineStr"/>
-      <c r="D92" s="4" t="inlineStr"/>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_MATRIX_RULES_INT</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr"/>
@@ -2790,11 +2998,19 @@
           <t>FA_MASSADD_DISTRIBUTIONS</t>
         </is>
       </c>
-      <c r="C111" s="4" t="inlineStr"/>
-      <c r="D111" s="4" t="inlineStr"/>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>T_FA_MASSADD_DISTRIBUTIONS</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>T66</t>
+        </is>
+      </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F111" s="4" t="inlineStr"/>
@@ -2811,11 +3027,19 @@
           <t>FA_MASS_ADDITIONS</t>
         </is>
       </c>
-      <c r="C112" s="4" t="inlineStr"/>
-      <c r="D112" s="4" t="inlineStr"/>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>T_FA_MASS_ADDITIONS</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>T65</t>
+        </is>
+      </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F112" s="4" t="inlineStr"/>
@@ -2932,11 +3156,19 @@
           <t>FA_RETIREMENTS_T</t>
         </is>
       </c>
-      <c r="C117" s="4" t="inlineStr"/>
-      <c r="D117" s="4" t="inlineStr"/>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>T_FA_RETIREMENTS_T</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>TE4</t>
+        </is>
+      </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F117" s="4" t="inlineStr"/>
@@ -4091,11 +4323,19 @@
           <t>INV_SERIAL_NUMBERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C172" s="4" t="inlineStr"/>
-      <c r="D172" s="4" t="inlineStr"/>
+      <c r="C172" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_SERIAL_NUMBERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>TK7</t>
+        </is>
+      </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F172" s="4" t="inlineStr"/>
@@ -4217,11 +4457,19 @@
           <t>CST_I_INCOMING_TXN_COSTS</t>
         </is>
       </c>
-      <c r="C178" s="4" t="inlineStr"/>
-      <c r="D178" s="4" t="inlineStr"/>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t>T_CST_I_INCOMING_TXN_COSTS</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>TG4</t>
+        </is>
+      </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F178" s="4" t="inlineStr"/>
@@ -4238,11 +4486,19 @@
           <t>INV_SERIAL_NUMBERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C179" s="4" t="inlineStr"/>
-      <c r="D179" s="4" t="inlineStr"/>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_SERIAL_NUMBERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>TK7</t>
+        </is>
+      </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F179" s="4" t="inlineStr"/>
@@ -4259,11 +4515,19 @@
           <t>INV_TRANSACTIONS_INTERFACE</t>
         </is>
       </c>
-      <c r="C180" s="4" t="inlineStr"/>
-      <c r="D180" s="4" t="inlineStr"/>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_TRANSACTIONS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>T47</t>
+        </is>
+      </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F180" s="4" t="inlineStr"/>
@@ -4343,11 +4607,19 @@
           <t>EGO_ITEM_INTF_EFF_B</t>
         </is>
       </c>
-      <c r="C184" s="4" t="inlineStr"/>
-      <c r="D184" s="4" t="inlineStr"/>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>T_EGO_ITEM_INTF_EFF_B</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>T86</t>
+        </is>
+      </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F184" s="4" t="inlineStr"/>
@@ -4490,11 +4762,19 @@
           <t>EGP_ITEM_ATTACHMENTS_INTF</t>
         </is>
       </c>
-      <c r="C191" s="4" t="inlineStr"/>
-      <c r="D191" s="4" t="inlineStr"/>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_ITEM_ATTACHMENTS_INTF</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t>T40</t>
+        </is>
+      </c>
       <c r="E191" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F191" s="4" t="inlineStr"/>
@@ -4553,11 +4833,19 @@
           <t>EGP_ITEM_RELATIONSHIPS_INTF</t>
         </is>
       </c>
-      <c r="C194" s="4" t="inlineStr"/>
-      <c r="D194" s="4" t="inlineStr"/>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_ITEM_RELATIONSHIPS_INTF</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>T88</t>
+        </is>
+      </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr"/>
@@ -4616,11 +4904,19 @@
           <t>EGP_SYSTEM_ITEMS_INTERFACE</t>
         </is>
       </c>
-      <c r="C197" s="4" t="inlineStr"/>
-      <c r="D197" s="4" t="inlineStr"/>
+      <c r="C197" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_SYSTEM_ITEMS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D197" s="4" t="inlineStr">
+        <is>
+          <t>T90</t>
+        </is>
+      </c>
       <c r="E197" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F197" s="4" t="inlineStr"/>
@@ -4691,11 +4987,19 @@
           <t>EGP_REF_DESGS_INTERFACE</t>
         </is>
       </c>
-      <c r="C200" s="4" t="inlineStr"/>
-      <c r="D200" s="4" t="inlineStr"/>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_REF_DESGS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>T93</t>
+        </is>
+      </c>
       <c r="E200" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F200" s="4" t="inlineStr"/>
@@ -4712,11 +5016,19 @@
           <t>EGP_STRUCTURES_INTERFACE</t>
         </is>
       </c>
-      <c r="C201" s="4" t="inlineStr"/>
-      <c r="D201" s="4" t="inlineStr"/>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_STRUCTURES_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>T94</t>
+        </is>
+      </c>
       <c r="E201" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F201" s="4" t="inlineStr"/>
@@ -4733,11 +5045,19 @@
           <t>EGP_SUB_COMPS_INTERFACE</t>
         </is>
       </c>
-      <c r="C202" s="4" t="inlineStr"/>
-      <c r="D202" s="4" t="inlineStr"/>
+      <c r="C202" s="4" t="inlineStr">
+        <is>
+          <t>T_EGP_SUB_COMPS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D202" s="4" t="inlineStr">
+        <is>
+          <t>T92</t>
+        </is>
+      </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr"/>
@@ -4754,15 +5074,27 @@
           <t>GL_INTERFACE</t>
         </is>
       </c>
-      <c r="C203" s="4" t="inlineStr"/>
-      <c r="D203" s="4" t="inlineStr"/>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>T_GL_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
       <c r="E203" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F203" s="4" t="inlineStr"/>
-      <c r="G203" s="5" t="inlineStr"/>
+      <c r="G203" s="5" t="inlineStr">
+        <is>
+          <t>Secondary prefix T02 (10 fields) also present</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
@@ -5867,11 +6199,19 @@
           <t>PO_HEADERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C256" s="4" t="inlineStr"/>
-      <c r="D256" s="4" t="inlineStr"/>
+      <c r="C256" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_HEADERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D256" s="4" t="inlineStr">
+        <is>
+          <t>T77</t>
+        </is>
+      </c>
       <c r="E256" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F256" s="4" t="inlineStr"/>
@@ -5888,11 +6228,19 @@
           <t>PO_LINES_INTERFACE</t>
         </is>
       </c>
-      <c r="C257" s="4" t="inlineStr"/>
-      <c r="D257" s="4" t="inlineStr"/>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_LINES_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>T79</t>
+        </is>
+      </c>
       <c r="E257" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F257" s="4" t="inlineStr"/>
@@ -5909,11 +6257,19 @@
           <t>PO_LINE_LOCATIONS_INTERFACE</t>
         </is>
       </c>
-      <c r="C258" s="4" t="inlineStr"/>
-      <c r="D258" s="4" t="inlineStr"/>
+      <c r="C258" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_LINE_LOCATIONS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D258" s="4" t="inlineStr">
+        <is>
+          <t>T78</t>
+        </is>
+      </c>
       <c r="E258" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F258" s="4" t="inlineStr"/>
@@ -5951,11 +6307,19 @@
           <t>PO_HEADERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C260" s="4" t="inlineStr"/>
-      <c r="D260" s="4" t="inlineStr"/>
+      <c r="C260" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_HEADERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D260" s="4" t="inlineStr">
+        <is>
+          <t>T77</t>
+        </is>
+      </c>
       <c r="E260" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F260" s="4" t="inlineStr"/>
@@ -6077,11 +6441,19 @@
           <t>PO_DISTRIBUTIONS_INTERFACE</t>
         </is>
       </c>
-      <c r="C266" s="4" t="inlineStr"/>
-      <c r="D266" s="4" t="inlineStr"/>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_DISTRIBUTIONS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr">
+        <is>
+          <t>T75</t>
+        </is>
+      </c>
       <c r="E266" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F266" s="4" t="inlineStr"/>
@@ -6098,11 +6470,19 @@
           <t>PO_HEADERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C267" s="4" t="inlineStr"/>
-      <c r="D267" s="4" t="inlineStr"/>
+      <c r="C267" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_HEADERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D267" s="4" t="inlineStr">
+        <is>
+          <t>T77</t>
+        </is>
+      </c>
       <c r="E267" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F267" s="4" t="inlineStr"/>
@@ -6119,11 +6499,19 @@
           <t>PO_LINES_INTERFACE</t>
         </is>
       </c>
-      <c r="C268" s="4" t="inlineStr"/>
-      <c r="D268" s="4" t="inlineStr"/>
+      <c r="C268" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_LINES_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D268" s="4" t="inlineStr">
+        <is>
+          <t>T79</t>
+        </is>
+      </c>
       <c r="E268" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F268" s="4" t="inlineStr"/>
@@ -6140,11 +6528,19 @@
           <t>PO_LINE_LOCATIONS_INTERFACE</t>
         </is>
       </c>
-      <c r="C269" s="4" t="inlineStr"/>
-      <c r="D269" s="4" t="inlineStr"/>
+      <c r="C269" s="4" t="inlineStr">
+        <is>
+          <t>T_PO_LINE_LOCATIONS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D269" s="4" t="inlineStr">
+        <is>
+          <t>T78</t>
+        </is>
+      </c>
       <c r="E269" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F269" s="4" t="inlineStr"/>
@@ -6203,11 +6599,19 @@
           <t>INV_LPN_INTERFACE</t>
         </is>
       </c>
-      <c r="C272" s="4" t="inlineStr"/>
-      <c r="D272" s="4" t="inlineStr"/>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_LPN_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D272" s="4" t="inlineStr">
+        <is>
+          <t>TK4</t>
+        </is>
+      </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F272" s="4" t="inlineStr"/>
@@ -6224,11 +6628,19 @@
           <t>INV_SERIAL_NUMBERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C273" s="4" t="inlineStr"/>
-      <c r="D273" s="4" t="inlineStr"/>
+      <c r="C273" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_SERIAL_NUMBERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D273" s="4" t="inlineStr">
+        <is>
+          <t>TK7</t>
+        </is>
+      </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F273" s="4" t="inlineStr"/>
@@ -6266,11 +6678,19 @@
           <t>WSH_FREIGHT_COSTS_INTERFACE</t>
         </is>
       </c>
-      <c r="C275" s="4" t="inlineStr"/>
-      <c r="D275" s="4" t="inlineStr"/>
+      <c r="C275" s="4" t="inlineStr">
+        <is>
+          <t>T_WSH_FREIGHT_COSTS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D275" s="4" t="inlineStr">
+        <is>
+          <t>TK8</t>
+        </is>
+      </c>
       <c r="E275" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F275" s="4" t="inlineStr"/>
@@ -6287,11 +6707,19 @@
           <t>WSH_NEW_DEL_INTERFACE</t>
         </is>
       </c>
-      <c r="C276" s="4" t="inlineStr"/>
-      <c r="D276" s="4" t="inlineStr"/>
+      <c r="C276" s="4" t="inlineStr">
+        <is>
+          <t>T_WSH_NEW_DEL_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D276" s="4" t="inlineStr">
+        <is>
+          <t>TK3</t>
+        </is>
+      </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F276" s="4" t="inlineStr"/>
@@ -6308,11 +6736,19 @@
           <t>WSH_SHIPMENT_LINE_INTERFACE</t>
         </is>
       </c>
-      <c r="C277" s="4" t="inlineStr"/>
-      <c r="D277" s="4" t="inlineStr"/>
+      <c r="C277" s="4" t="inlineStr">
+        <is>
+          <t>T_WSH_SHIPMENT_LINE_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>TK5</t>
+        </is>
+      </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F277" s="4" t="inlineStr"/>
@@ -6560,11 +6996,19 @@
           <t>QP_MATRIX_DIMENSIONS_INT</t>
         </is>
       </c>
-      <c r="C289" s="4" t="inlineStr"/>
-      <c r="D289" s="4" t="inlineStr"/>
+      <c r="C289" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_MATRIX_DIMENSIONS_INT</t>
+        </is>
+      </c>
+      <c r="D289" s="4" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F289" s="4" t="inlineStr"/>
@@ -6581,11 +7025,19 @@
           <t>QP_MATRIX_RULES_INT</t>
         </is>
       </c>
-      <c r="C290" s="4" t="inlineStr"/>
-      <c r="D290" s="4" t="inlineStr"/>
+      <c r="C290" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_MATRIX_RULES_INT</t>
+        </is>
+      </c>
+      <c r="D290" s="4" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F290" s="4" t="inlineStr"/>
@@ -6602,11 +7054,19 @@
           <t>QP_PL_COMP_ITEMS_INT</t>
         </is>
       </c>
-      <c r="C291" s="4" t="inlineStr"/>
-      <c r="D291" s="4" t="inlineStr"/>
+      <c r="C291" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_PL_COMP_ITEMS_INT</t>
+        </is>
+      </c>
+      <c r="D291" s="4" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F291" s="4" t="inlineStr"/>
@@ -6644,11 +7104,19 @@
           <t>QP_PRICE_LISTS_INT</t>
         </is>
       </c>
-      <c r="C293" s="4" t="inlineStr"/>
-      <c r="D293" s="4" t="inlineStr"/>
+      <c r="C293" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_PRICE_LISTS_INT</t>
+        </is>
+      </c>
+      <c r="D293" s="4" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F293" s="4" t="inlineStr"/>
@@ -6665,11 +7133,19 @@
           <t>QP_PRICE_LIST_CHARGES_INT</t>
         </is>
       </c>
-      <c r="C294" s="4" t="inlineStr"/>
-      <c r="D294" s="4" t="inlineStr"/>
+      <c r="C294" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_PRICE_LIST_CHARGES_INT</t>
+        </is>
+      </c>
+      <c r="D294" s="4" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F294" s="4" t="inlineStr"/>
@@ -6686,11 +7162,19 @@
           <t>QP_PRICE_LIST_ITEMS_INT</t>
         </is>
       </c>
-      <c r="C295" s="4" t="inlineStr"/>
-      <c r="D295" s="4" t="inlineStr"/>
+      <c r="C295" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_PRICE_LIST_ITEMS_INT</t>
+        </is>
+      </c>
+      <c r="D295" s="4" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F295" s="4" t="inlineStr"/>
@@ -6707,11 +7191,19 @@
           <t>QP_PRICE_LIST_SETS_INT</t>
         </is>
       </c>
-      <c r="C296" s="4" t="inlineStr"/>
-      <c r="D296" s="4" t="inlineStr"/>
+      <c r="C296" s="4" t="inlineStr">
+        <is>
+          <t>T_QP_PRICE_LIST_SETS_INT</t>
+        </is>
+      </c>
+      <c r="D296" s="4" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F296" s="4" t="inlineStr"/>
@@ -7538,11 +8030,19 @@
           <t>PJO_BUDGETS_XFACE</t>
         </is>
       </c>
-      <c r="C335" s="4" t="inlineStr"/>
-      <c r="D335" s="4" t="inlineStr"/>
+      <c r="C335" s="4" t="inlineStr">
+        <is>
+          <t>T_PJO_BUDGETS_XFACE</t>
+        </is>
+      </c>
+      <c r="D335" s="4" t="inlineStr">
+        <is>
+          <t>T54</t>
+        </is>
+      </c>
       <c r="E335" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F335" s="4" t="inlineStr"/>
@@ -8147,11 +8647,19 @@
           <t>PJF_PROJ_ELEMENTS_XFACE</t>
         </is>
       </c>
-      <c r="C364" s="4" t="inlineStr"/>
-      <c r="D364" s="4" t="inlineStr"/>
+      <c r="C364" s="4" t="inlineStr">
+        <is>
+          <t>T_PJF_PROJ_ELEMENTS_XFACE</t>
+        </is>
+      </c>
+      <c r="D364" s="4" t="inlineStr">
+        <is>
+          <t>T53</t>
+        </is>
+      </c>
       <c r="E364" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F364" s="4" t="inlineStr"/>
@@ -8189,11 +8697,19 @@
           <t>PJC_TXN_XFACE_STAGE_ALL</t>
         </is>
       </c>
-      <c r="C366" s="4" t="inlineStr"/>
-      <c r="D366" s="4" t="inlineStr"/>
+      <c r="C366" s="4" t="inlineStr">
+        <is>
+          <t>T_PJC_TXN_XFACE_STAGE_ALL</t>
+        </is>
+      </c>
+      <c r="D366" s="4" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
       <c r="E366" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F366" s="4" t="inlineStr"/>
@@ -8210,11 +8726,19 @@
           <t>PJC_TXN_XFACE_STAGE_ALL</t>
         </is>
       </c>
-      <c r="C367" s="4" t="inlineStr"/>
-      <c r="D367" s="4" t="inlineStr"/>
+      <c r="C367" s="4" t="inlineStr">
+        <is>
+          <t>T_PJC_TXN_XFACE_STAGE_ALL</t>
+        </is>
+      </c>
+      <c r="D367" s="4" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
       <c r="E367" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F367" s="4" t="inlineStr"/>
@@ -8231,11 +8755,19 @@
           <t>PJC_TXN_XFACE_STAGE_ALL</t>
         </is>
       </c>
-      <c r="C368" s="4" t="inlineStr"/>
-      <c r="D368" s="4" t="inlineStr"/>
+      <c r="C368" s="4" t="inlineStr">
+        <is>
+          <t>T_PJC_TXN_XFACE_STAGE_ALL</t>
+        </is>
+      </c>
+      <c r="D368" s="4" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
       <c r="E368" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F368" s="4" t="inlineStr"/>
@@ -8252,11 +8784,19 @@
           <t>PJC_TXN_XFACE_STAGE_ALL</t>
         </is>
       </c>
-      <c r="C369" s="4" t="inlineStr"/>
-      <c r="D369" s="4" t="inlineStr"/>
+      <c r="C369" s="4" t="inlineStr">
+        <is>
+          <t>T_PJC_TXN_XFACE_STAGE_ALL</t>
+        </is>
+      </c>
+      <c r="D369" s="4" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
       <c r="E369" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F369" s="4" t="inlineStr"/>
@@ -8273,11 +8813,19 @@
           <t>PJC_TXN_XFACE_STAGE_ALL</t>
         </is>
       </c>
-      <c r="C370" s="4" t="inlineStr"/>
-      <c r="D370" s="4" t="inlineStr"/>
+      <c r="C370" s="4" t="inlineStr">
+        <is>
+          <t>T_PJC_TXN_XFACE_STAGE_ALL</t>
+        </is>
+      </c>
+      <c r="D370" s="4" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
       <c r="E370" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F370" s="4" t="inlineStr"/>
@@ -8294,11 +8842,19 @@
           <t>PJC_TXN_XFACE_STAGE_ALL</t>
         </is>
       </c>
-      <c r="C371" s="4" t="inlineStr"/>
-      <c r="D371" s="4" t="inlineStr"/>
+      <c r="C371" s="4" t="inlineStr">
+        <is>
+          <t>T_PJC_TXN_XFACE_STAGE_ALL</t>
+        </is>
+      </c>
+      <c r="D371" s="4" t="inlineStr">
+        <is>
+          <t>T39</t>
+        </is>
+      </c>
       <c r="E371" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F371" s="4" t="inlineStr"/>
@@ -8600,11 +9156,19 @@
           <t>INV_LPN_INTERFACE</t>
         </is>
       </c>
-      <c r="C385" s="4" t="inlineStr"/>
-      <c r="D385" s="4" t="inlineStr"/>
+      <c r="C385" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_LPN_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D385" s="4" t="inlineStr">
+        <is>
+          <t>TK4</t>
+        </is>
+      </c>
       <c r="E385" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F385" s="4" t="inlineStr"/>
@@ -8621,11 +9185,19 @@
           <t>INV_SERIAL_NUMBERS_INTERFACE</t>
         </is>
       </c>
-      <c r="C386" s="4" t="inlineStr"/>
-      <c r="D386" s="4" t="inlineStr"/>
+      <c r="C386" s="4" t="inlineStr">
+        <is>
+          <t>T_INV_SERIAL_NUMBERS_INTERFACE</t>
+        </is>
+      </c>
+      <c r="D386" s="4" t="inlineStr">
+        <is>
+          <t>TK7</t>
+        </is>
+      </c>
       <c r="E386" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F386" s="4" t="inlineStr"/>
@@ -11589,11 +12161,19 @@
           <t>DOO_ORDER_ADDRESSES_INT</t>
         </is>
       </c>
-      <c r="C526" s="4" t="inlineStr"/>
-      <c r="D526" s="4" t="inlineStr"/>
+      <c r="C526" s="4" t="inlineStr">
+        <is>
+          <t>T_DOO_ORDER_ADDRESSES_INT</t>
+        </is>
+      </c>
+      <c r="D526" s="4" t="inlineStr">
+        <is>
+          <t>TB9</t>
+        </is>
+      </c>
       <c r="E526" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F526" s="4" t="inlineStr"/>
@@ -11631,11 +12211,19 @@
           <t>DOO_ORDER_CHARGES_INT</t>
         </is>
       </c>
-      <c r="C528" s="4" t="inlineStr"/>
-      <c r="D528" s="4" t="inlineStr"/>
+      <c r="C528" s="4" t="inlineStr">
+        <is>
+          <t>T_DOO_ORDER_CHARGES_INT</t>
+        </is>
+      </c>
+      <c r="D528" s="4" t="inlineStr">
+        <is>
+          <t>TC2</t>
+        </is>
+      </c>
       <c r="E528" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F528" s="4" t="inlineStr"/>
@@ -12075,11 +12663,19 @@
           <t>IBY_TEMP_EXT_PAYEES</t>
         </is>
       </c>
-      <c r="C548" s="4" t="inlineStr"/>
-      <c r="D548" s="4" t="inlineStr"/>
+      <c r="C548" s="4" t="inlineStr">
+        <is>
+          <t>T_IBY_TEMP_EXT_PAYEES</t>
+        </is>
+      </c>
+      <c r="D548" s="4" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
       <c r="E548" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F548" s="4" t="inlineStr"/>
@@ -12096,11 +12692,19 @@
           <t>IBY_TEMP_PMT_INSTR_USES</t>
         </is>
       </c>
-      <c r="C549" s="4" t="inlineStr"/>
-      <c r="D549" s="4" t="inlineStr"/>
+      <c r="C549" s="4" t="inlineStr">
+        <is>
+          <t>T_IBY_TEMP_PMT_INSTR_USES</t>
+        </is>
+      </c>
+      <c r="D549" s="4" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
       <c r="E549" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F549" s="4" t="inlineStr"/>
@@ -12117,11 +12721,19 @@
           <t>POZ_SUP_BUS_CLASS_INT</t>
         </is>
       </c>
-      <c r="C550" s="4" t="inlineStr"/>
-      <c r="D550" s="4" t="inlineStr"/>
+      <c r="C550" s="4" t="inlineStr">
+        <is>
+          <t>T_POZ_SUP_BUS_CLASS_INT</t>
+        </is>
+      </c>
+      <c r="D550" s="4" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
       <c r="E550" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F550" s="4" t="inlineStr"/>
@@ -12180,11 +12792,19 @@
           <t>POZ_SUPPLIERS_INT</t>
         </is>
       </c>
-      <c r="C553" s="4" t="inlineStr"/>
-      <c r="D553" s="4" t="inlineStr"/>
+      <c r="C553" s="4" t="inlineStr">
+        <is>
+          <t>T_POZ_SUPPLIERS_INT</t>
+        </is>
+      </c>
+      <c r="D553" s="4" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
       <c r="E553" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F553" s="4" t="inlineStr"/>
@@ -12222,11 +12842,19 @@
           <t>POZ_SITE_ASSIGNMENTS_INT</t>
         </is>
       </c>
-      <c r="C555" s="4" t="inlineStr"/>
-      <c r="D555" s="4" t="inlineStr"/>
+      <c r="C555" s="4" t="inlineStr">
+        <is>
+          <t>T_POZ_SITE_ASSIGNMENTS_INT</t>
+        </is>
+      </c>
+      <c r="D555" s="4" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
       <c r="E555" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="F555" s="4" t="inlineStr"/>

</xml_diff>